<commit_message>
chore: update excel generation to include Tasarim_Sablonlari mappings
</commit_message>
<xml_diff>
--- a/Derslig_Tisho_Varyant_Katalogu.xlsx
+++ b/Derslig_Tisho_Varyant_Katalogu.xlsx
@@ -5608,7 +5608,22 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M11"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="60.83203125" customWidth="1"/>
+    <col min="8" max="8" width="60.83203125" customWidth="1"/>
+    <col min="9" max="9" width="8.83203125" customWidth="1"/>
+    <col min="10" max="10" width="8.83203125" customWidth="1"/>
+    <col min="11" max="11" width="8.83203125" customWidth="1"/>
+    <col min="12" max="12" width="8.83203125" customWidth="1"/>
+    <col min="13" max="13" width="8.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5653,16 +5668,16 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>888721</v>
+        <v>101</v>
       </c>
       <c r="B2" t="str">
-        <v>Matematik Dehasi</v>
+        <v>Teacher Mode OFF</v>
       </c>
       <c r="C2" t="str">
-        <v>koyu</v>
+        <v>Koyu</v>
       </c>
       <c r="D2" t="str">
-        <v>Beyaz tisort</v>
+        <v>Beyaz</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -5671,10 +5686,10 @@
         <v>photo</v>
       </c>
       <c r="G2" t="str">
-        <v>https://derslig.com/designs/d1-dark-front.png</v>
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_teachermode_beyaz.png</v>
       </c>
       <c r="H2" t="str">
-        <v>https://derslig.com/designs/d1-dark-front-big.png</v>
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_teachermode_beyaz.png</v>
       </c>
       <c r="I2">
         <v>120</v>
@@ -5692,11 +5707,378 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3">
+        <v>102</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Teacher Mode OFF</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Acik</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Siyah</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="str">
+        <v>photo</v>
+      </c>
+      <c r="G3" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_teachermode_siyah.png</v>
+      </c>
+      <c r="H3" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_teachermode_siyah.png</v>
+      </c>
+      <c r="I3">
+        <v>120</v>
+      </c>
+      <c r="J3">
+        <v>80</v>
+      </c>
+      <c r="K3">
+        <v>300</v>
+      </c>
+      <c r="L3">
+        <v>400</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>201</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Tatil Hesabı</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Koyu</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Beyaz</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v>photo</v>
+      </c>
+      <c r="G4" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_2ay3ay_beyaz.png</v>
+      </c>
+      <c r="H4" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_2ay3ay_beyaz.png</v>
+      </c>
+      <c r="I4">
+        <v>120</v>
+      </c>
+      <c r="J4">
+        <v>80</v>
+      </c>
+      <c r="K4">
+        <v>300</v>
+      </c>
+      <c r="L4">
+        <v>400</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>202</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Tatil Hesabı</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Acik</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Siyah</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v>photo</v>
+      </c>
+      <c r="G5" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_2ay3ay_siyah.png</v>
+      </c>
+      <c r="H5" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_2ay3ay_siyah.png</v>
+      </c>
+      <c r="I5">
+        <v>120</v>
+      </c>
+      <c r="J5">
+        <v>80</v>
+      </c>
+      <c r="K5">
+        <v>300</v>
+      </c>
+      <c r="L5">
+        <v>400</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>301</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Gergin Yay</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Koyu</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Beyaz</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v>photo</v>
+      </c>
+      <c r="G6" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_gerginyay_beyaz.png</v>
+      </c>
+      <c r="H6" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_gerginyay_beyaz.png</v>
+      </c>
+      <c r="I6">
+        <v>120</v>
+      </c>
+      <c r="J6">
+        <v>80</v>
+      </c>
+      <c r="K6">
+        <v>300</v>
+      </c>
+      <c r="L6">
+        <v>400</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>302</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Gergin Yay</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Acik</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Siyah</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" t="str">
+        <v>photo</v>
+      </c>
+      <c r="G7" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_gerginyay_siyah.png</v>
+      </c>
+      <c r="H7" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_gerginyay_siyah.png</v>
+      </c>
+      <c r="I7">
+        <v>120</v>
+      </c>
+      <c r="J7">
+        <v>80</v>
+      </c>
+      <c r="K7">
+        <v>300</v>
+      </c>
+      <c r="L7">
+        <v>400</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>401</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Renkli Matematik</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Koyu</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Beyaz</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" t="str">
+        <v>photo</v>
+      </c>
+      <c r="G8" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_teacher_beyaz.png</v>
+      </c>
+      <c r="H8" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_teacher_beyaz.png</v>
+      </c>
+      <c r="I8">
+        <v>120</v>
+      </c>
+      <c r="J8">
+        <v>80</v>
+      </c>
+      <c r="K8">
+        <v>300</v>
+      </c>
+      <c r="L8">
+        <v>400</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>402</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Renkli Matematik</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Acik</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Siyah</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9" t="str">
+        <v>photo</v>
+      </c>
+      <c r="G9" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_teacher_siyah.png</v>
+      </c>
+      <c r="H9" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_teacher_siyah.png</v>
+      </c>
+      <c r="I9">
+        <v>120</v>
+      </c>
+      <c r="J9">
+        <v>80</v>
+      </c>
+      <c r="K9">
+        <v>300</v>
+      </c>
+      <c r="L9">
+        <v>400</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>501</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Tatil Modu</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Koyu</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Beyaz</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10" t="str">
+        <v>photo</v>
+      </c>
+      <c r="G10" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_tatilmodu_beyaz.png</v>
+      </c>
+      <c r="H10" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_tatilmodu_beyaz.png</v>
+      </c>
+      <c r="I10">
+        <v>120</v>
+      </c>
+      <c r="J10">
+        <v>80</v>
+      </c>
+      <c r="K10">
+        <v>300</v>
+      </c>
+      <c r="L10">
+        <v>400</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>502</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Tatil Modu</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Acik</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Siyah</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11" t="str">
+        <v>photo</v>
+      </c>
+      <c r="G11" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_tatilmodu_siyah.png</v>
+      </c>
+      <c r="H11" t="str">
+        <v>https://onurkaya-ai.github.io/derslig-maarif/landing_assets/design_tatilmodu_siyah.png</v>
+      </c>
+      <c r="I11">
+        <v>120</v>
+      </c>
+      <c r="J11">
+        <v>80</v>
+      </c>
+      <c r="K11">
+        <v>300</v>
+      </c>
+      <c r="L11">
+        <v>400</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M2"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: append tisho design links to excel generator
</commit_message>
<xml_diff>
--- a/Derslig_Tisho_Varyant_Katalogu.xlsx
+++ b/Derslig_Tisho_Varyant_Katalogu.xlsx
@@ -529,7 +529,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P101"/>
+  <dimension ref="A1:Q101"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -547,6 +547,7 @@
     <col min="14" max="14" width="10.83203125" customWidth="1"/>
     <col min="15" max="15" width="15.83203125" customWidth="1"/>
     <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -598,6 +599,9 @@
       <c r="P1" t="str">
         <v>not</v>
       </c>
+      <c r="Q1" t="str">
+        <v>tisho_tasarim_link</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -648,6 +652,9 @@
       <c r="P2" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q2" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -698,6 +705,9 @@
       <c r="P3" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q3" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -748,6 +758,9 @@
       <c r="P4" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q4" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -798,6 +811,9 @@
       <c r="P5" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q5" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -848,6 +864,9 @@
       <c r="P6" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q6" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -898,6 +917,9 @@
       <c r="P7" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q7" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -948,6 +970,9 @@
       <c r="P8" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q8" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -998,6 +1023,9 @@
       <c r="P9" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q9" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -1048,6 +1076,9 @@
       <c r="P10" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q10" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -1098,6 +1129,9 @@
       <c r="P11" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q11" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1148,6 +1182,9 @@
       <c r="P12" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q12" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee158af5b46ee015c2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1198,6 +1235,9 @@
       <c r="P13" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q13" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee158af5b46ee015c2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1248,6 +1288,9 @@
       <c r="P14" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q14" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee158af5b46ee015c2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1298,6 +1341,9 @@
       <c r="P15" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q15" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee158af5b46ee015c2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1348,6 +1394,9 @@
       <c r="P16" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q16" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee158af5b46ee015c2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1398,6 +1447,9 @@
       <c r="P17" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q17" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1448,6 +1500,9 @@
       <c r="P18" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q18" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1498,6 +1553,9 @@
       <c r="P19" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q19" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1548,6 +1606,9 @@
       <c r="P20" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q20" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1598,6 +1659,9 @@
       <c r="P21" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q21" t="str">
+        <v>https://www.tisho.com/tasarim#getDesign=19ee1582bdce7e74d162</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1648,6 +1712,9 @@
       <c r="P22" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1698,6 +1765,9 @@
       <c r="P23" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1748,6 +1818,9 @@
       <c r="P24" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1798,6 +1871,9 @@
       <c r="P25" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1848,6 +1924,9 @@
       <c r="P26" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1898,6 +1977,9 @@
       <c r="P27" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1948,6 +2030,9 @@
       <c r="P28" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1998,6 +2083,9 @@
       <c r="P29" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -2048,6 +2136,9 @@
       <c r="P30" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -2098,6 +2189,9 @@
       <c r="P31" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -2148,6 +2242,9 @@
       <c r="P32" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -2198,6 +2295,9 @@
       <c r="P33" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2248,6 +2348,9 @@
       <c r="P34" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2298,6 +2401,9 @@
       <c r="P35" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -2348,6 +2454,9 @@
       <c r="P36" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2398,6 +2507,9 @@
       <c r="P37" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -2448,6 +2560,9 @@
       <c r="P38" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -2498,6 +2613,9 @@
       <c r="P39" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -2548,6 +2666,9 @@
       <c r="P40" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2598,6 +2719,9 @@
       <c r="P41" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -2648,6 +2772,9 @@
       <c r="P42" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2698,6 +2825,9 @@
       <c r="P43" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -2748,6 +2878,9 @@
       <c r="P44" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2798,6 +2931,9 @@
       <c r="P45" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2848,6 +2984,9 @@
       <c r="P46" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2898,6 +3037,9 @@
       <c r="P47" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2948,6 +3090,9 @@
       <c r="P48" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2998,6 +3143,9 @@
       <c r="P49" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -3048,6 +3196,9 @@
       <c r="P50" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -3098,6 +3249,9 @@
       <c r="P51" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -3148,6 +3302,9 @@
       <c r="P52" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -3198,6 +3355,9 @@
       <c r="P53" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -3248,6 +3408,9 @@
       <c r="P54" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -3298,6 +3461,9 @@
       <c r="P55" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -3348,6 +3514,9 @@
       <c r="P56" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -3398,6 +3567,9 @@
       <c r="P57" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -3448,6 +3620,9 @@
       <c r="P58" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -3498,6 +3673,9 @@
       <c r="P59" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -3548,6 +3726,9 @@
       <c r="P60" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -3598,6 +3779,9 @@
       <c r="P61" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -3648,6 +3832,9 @@
       <c r="P62" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -3698,6 +3885,9 @@
       <c r="P63" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -3748,6 +3938,9 @@
       <c r="P64" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -3798,6 +3991,9 @@
       <c r="P65" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -3848,6 +4044,9 @@
       <c r="P66" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -3898,6 +4097,9 @@
       <c r="P67" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -3948,6 +4150,9 @@
       <c r="P68" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -3998,6 +4203,9 @@
       <c r="P69" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -4048,6 +4256,9 @@
       <c r="P70" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -4098,6 +4309,9 @@
       <c r="P71" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -4148,6 +4362,9 @@
       <c r="P72" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -4198,6 +4415,9 @@
       <c r="P73" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -4248,6 +4468,9 @@
       <c r="P74" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -4298,6 +4521,9 @@
       <c r="P75" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -4348,6 +4574,9 @@
       <c r="P76" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -4398,6 +4627,9 @@
       <c r="P77" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -4448,6 +4680,9 @@
       <c r="P78" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -4498,6 +4733,9 @@
       <c r="P79" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -4548,6 +4786,9 @@
       <c r="P80" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -4598,6 +4839,9 @@
       <c r="P81" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -4648,6 +4892,9 @@
       <c r="P82" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -4698,6 +4945,9 @@
       <c r="P83" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -4748,6 +4998,9 @@
       <c r="P84" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -4798,6 +5051,9 @@
       <c r="P85" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -4848,6 +5104,9 @@
       <c r="P86" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -4898,6 +5157,9 @@
       <c r="P87" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -4948,6 +5210,9 @@
       <c r="P88" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -4998,6 +5263,9 @@
       <c r="P89" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -5048,6 +5316,9 @@
       <c r="P90" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -5098,6 +5369,9 @@
       <c r="P91" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -5148,6 +5422,9 @@
       <c r="P92" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -5198,6 +5475,9 @@
       <c r="P93" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -5248,6 +5528,9 @@
       <c r="P94" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -5298,6 +5581,9 @@
       <c r="P95" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q95" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -5348,6 +5634,9 @@
       <c r="P96" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q96" t="str">
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -5398,6 +5687,9 @@
       <c r="P97" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q97" t="str">
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -5448,6 +5740,9 @@
       <c r="P98" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q98" t="str">
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -5498,6 +5793,9 @@
       <c r="P99" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q99" t="str">
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -5548,6 +5846,9 @@
       <c r="P100" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q100" t="str">
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -5598,10 +5899,13 @@
       <c r="P101" t="str">
         <v>Otomatik dolduruldu</v>
       </c>
+      <c r="Q101" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q101"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>